<commit_message>
obbbafim forecast sheet - part 5
final changes
</commit_message>
<xml_diff>
--- a/results/07-2025/beta/contributions-07-2025.xlsx
+++ b/results/07-2025/beta/contributions-07-2025.xlsx
@@ -22259,7 +22259,7 @@
         <v>0</v>
       </c>
       <c r="D223" t="n">
-        <v>-0.250199510132909</v>
+        <v>-0.218091441390802</v>
       </c>
       <c r="E223" t="n">
         <v>-0.199879916241108</v>
@@ -22316,13 +22316,13 @@
         <v>-0.00151505975298941</v>
       </c>
       <c r="W223" t="n">
-        <v>0.243428195800901</v>
+        <v>0.242347826012976</v>
       </c>
       <c r="X223" t="n">
-        <v>-0.00627217178817736</v>
+        <v>-0.00677250107663066</v>
       </c>
       <c r="Y223" t="n">
-        <v>-0.452964229106557</v>
+        <v>-0.420856160364451</v>
       </c>
       <c r="Z223" t="n">
         <v>0.00288480273254083</v>
@@ -22331,16 +22331,16 @@
         <v>-0.088289444952879</v>
       </c>
       <c r="AB223" t="n">
-        <v>0.136614390202252</v>
+        <v>0.135033221417888</v>
       </c>
       <c r="AC223" t="n">
-        <v>-0.951548611628606</v>
+        <v>-0.953131244205811</v>
       </c>
       <c r="AD223" t="n">
-        <v>-1.40162803800262</v>
+        <v>-1.37110260183772</v>
       </c>
       <c r="AE223" t="n">
-        <v>-0.265403650799482</v>
+        <v>-0.257772291758256</v>
       </c>
     </row>
     <row r="224">
@@ -22354,7 +22354,7 @@
         <v>0</v>
       </c>
       <c r="D224" t="n">
-        <v>-0.166032314733355</v>
+        <v>-0.166335102426299</v>
       </c>
       <c r="E224" t="n">
         <v>-0.188402753588166</v>
@@ -22366,7 +22366,7 @@
         <v>-0.00499532512598115</v>
       </c>
       <c r="H224" t="n">
-        <v>-0.0395148927973874</v>
+        <v>0.141866401137088</v>
       </c>
       <c r="I224" t="n">
         <v>0.185730312532247</v>
@@ -22411,31 +22411,31 @@
         <v>-0.000451773171946533</v>
       </c>
       <c r="W224" t="n">
-        <v>0.172464448233597</v>
+        <v>0.170312754424817</v>
       </c>
       <c r="X224" t="n">
-        <v>0.0167197530513641</v>
+        <v>0.0157297326996495</v>
       </c>
       <c r="Y224" t="n">
-        <v>-0.219157634022844</v>
+        <v>-0.219460421715788</v>
       </c>
       <c r="Z224" t="n">
         <v>-0.135277434298677</v>
       </c>
       <c r="AA224" t="n">
-        <v>0.104538323808508</v>
+        <v>0.285644148739794</v>
       </c>
       <c r="AB224" t="n">
-        <v>0.121299413270645</v>
+        <v>0.118157605258083</v>
       </c>
       <c r="AC224" t="n">
-        <v>-0.774296001511843</v>
+        <v>-0.596554324326954</v>
       </c>
       <c r="AD224" t="n">
-        <v>-1.12873106983336</v>
+        <v>-0.951292180341419</v>
       </c>
       <c r="AE224" t="n">
-        <v>-0.672944430770533</v>
+        <v>-0.620953349356321</v>
       </c>
     </row>
     <row r="225">
@@ -22449,7 +22449,7 @@
         <v>0</v>
       </c>
       <c r="D225" t="n">
-        <v>0.0253758993631041</v>
+        <v>0.138347808668163</v>
       </c>
       <c r="E225" t="n">
         <v>-0.187426688324483</v>
@@ -22461,7 +22461,7 @@
         <v>-0.0153552438046491</v>
       </c>
       <c r="H225" t="n">
-        <v>-0.0358643867623123</v>
+        <v>0.140377254322351</v>
       </c>
       <c r="I225" t="n">
         <v>0.0729643688673298</v>
@@ -22470,7 +22470,7 @@
         <v>0.00545401864232233</v>
       </c>
       <c r="K225" t="n">
-        <v>-0.0186080156825595</v>
+        <v>-0.0366943534705917</v>
       </c>
       <c r="L225" t="n">
         <v>0.0314648671659881</v>
@@ -22506,31 +22506,31 @@
         <v>-0.000419227109622843</v>
       </c>
       <c r="W225" t="n">
-        <v>0.121072944906745</v>
+        <v>0.129494712030853</v>
       </c>
       <c r="X225" t="n">
-        <v>0.033558144442533</v>
+        <v>0.0374417781397447</v>
       </c>
       <c r="Y225" t="n">
-        <v>-0.080169532365765</v>
+        <v>0.0328023769392936</v>
       </c>
       <c r="Z225" t="n">
         <v>-0.0818812565956142</v>
       </c>
       <c r="AA225" t="n">
-        <v>0.0215189867322611</v>
+        <v>0.197653824473987</v>
       </c>
       <c r="AB225" t="n">
-        <v>0.0906350601298607</v>
+        <v>0.0848773632426025</v>
       </c>
       <c r="AC225" t="n">
-        <v>-0.88786655633996</v>
+        <v>-0.717646085911434</v>
       </c>
       <c r="AD225" t="n">
-        <v>-1.04991734530134</v>
+        <v>-0.766724965567754</v>
       </c>
       <c r="AE225" t="n">
-        <v>-1.02334708307678</v>
+        <v>-0.900557906729174</v>
       </c>
     </row>
     <row r="226">
@@ -22544,19 +22544,19 @@
         <v>0</v>
       </c>
       <c r="D226" t="n">
-        <v>-0.149403326737253</v>
+        <v>0.182123494913557</v>
       </c>
       <c r="E226" t="n">
         <v>-0.186244865759511</v>
       </c>
       <c r="F226" t="n">
-        <v>0.306590654627882</v>
+        <v>0.141087528212335</v>
       </c>
       <c r="G226" t="n">
         <v>-0.0206587577015947</v>
       </c>
       <c r="H226" t="n">
-        <v>-0.0215016380398408</v>
+        <v>0.0352176317081096</v>
       </c>
       <c r="I226" t="n">
         <v>0.316467212868588</v>
@@ -22565,7 +22565,7 @@
         <v>0.00364314963120222</v>
       </c>
       <c r="K226" t="n">
-        <v>-0.163729181568732</v>
+        <v>-0.175460839059818</v>
       </c>
       <c r="L226" t="n">
         <v>0.0385868919646275</v>
@@ -22601,31 +22601,31 @@
         <v>-0.000388464898983852</v>
       </c>
       <c r="W226" t="n">
-        <v>0.116596252482861</v>
+        <v>0.135514231959327</v>
       </c>
       <c r="X226" t="n">
-        <v>-0.0136242291221517</v>
+        <v>-0.00480605503782594</v>
       </c>
       <c r="Y226" t="n">
-        <v>-0.201939285491737</v>
+        <v>0.129587536159072</v>
       </c>
       <c r="Z226" t="n">
         <v>-0.133708907005026</v>
       </c>
       <c r="AA226" t="n">
-        <v>0.583762092627697</v>
+        <v>0.475201884951763</v>
       </c>
       <c r="AB226" t="n">
-        <v>-0.0661469008035539</v>
+        <v>-0.0500870100151668</v>
       </c>
       <c r="AC226" t="n">
-        <v>-0.481975077553002</v>
+        <v>-0.574632611434394</v>
       </c>
       <c r="AD226" t="n">
-        <v>-0.817623270049766</v>
+        <v>-0.578753982280349</v>
       </c>
       <c r="AE226" t="n">
-        <v>-1.09947493079677</v>
+        <v>-0.916968432506811</v>
       </c>
     </row>
     <row r="227">
@@ -22639,19 +22639,19 @@
         <v>0</v>
       </c>
       <c r="D227" t="n">
-        <v>-0.150854113272481</v>
+        <v>-0.091179211129241</v>
       </c>
       <c r="E227" t="n">
         <v>-0.197303734077729</v>
       </c>
       <c r="F227" t="n">
-        <v>0.277658697237849</v>
+        <v>0.114356039802799</v>
       </c>
       <c r="G227" t="n">
         <v>-0.00901379205779021</v>
       </c>
       <c r="H227" t="n">
-        <v>-0.0222887098182955</v>
+        <v>0.0330798926987005</v>
       </c>
       <c r="I227" t="n">
         <v>0.251039235479208</v>
@@ -22660,7 +22660,7 @@
         <v>0.00487621229521312</v>
       </c>
       <c r="K227" t="n">
-        <v>-0.163385782850788</v>
+        <v>-0.168986483119721</v>
       </c>
       <c r="L227" t="n">
         <v>0.0110356741019841</v>
@@ -22696,31 +22696,31 @@
         <v>-0.000339139413338695</v>
       </c>
       <c r="W227" t="n">
-        <v>0.047091497868414</v>
+        <v>0.0952519114350495</v>
       </c>
       <c r="X227" t="n">
-        <v>0.0203155642193202</v>
+        <v>0.0168723614178661</v>
       </c>
       <c r="Y227" t="n">
-        <v>-0.236149513539501</v>
+        <v>-0.176474611396261</v>
       </c>
       <c r="Z227" t="n">
         <v>-0.11200833381071</v>
       </c>
       <c r="AA227" t="n">
-        <v>0.501680247177725</v>
+        <v>0.393923358464019</v>
       </c>
       <c r="AB227" t="n">
-        <v>-0.118160783171558</v>
+        <v>-0.0789579260105366</v>
       </c>
       <c r="AC227" t="n">
-        <v>0.384147573811116</v>
+        <v>0.315294958430772</v>
       </c>
       <c r="AD227" t="n">
-        <v>0.0359897264609053</v>
+        <v>0.0268120132238019</v>
       </c>
       <c r="AE227" t="n">
-        <v>-0.740070489680891</v>
+        <v>-0.56748977874143</v>
       </c>
     </row>
     <row r="228">
@@ -22734,19 +22734,19 @@
         <v>0</v>
       </c>
       <c r="D228" t="n">
-        <v>-0.142450451880153</v>
+        <v>-0.0711419432935427</v>
       </c>
       <c r="E228" t="n">
         <v>-0.187119724943941</v>
       </c>
       <c r="F228" t="n">
-        <v>0.151678303472226</v>
+        <v>0.0724111854320921</v>
       </c>
       <c r="G228" t="n">
         <v>0.00509242029859333</v>
       </c>
       <c r="H228" t="n">
-        <v>-0.0103979632781975</v>
+        <v>0.0432668687960049</v>
       </c>
       <c r="I228" t="n">
         <v>0.0775952242339403</v>
@@ -22755,7 +22755,7 @@
         <v>0.00640109336423803</v>
       </c>
       <c r="K228" t="n">
-        <v>-0.163850551205058</v>
+        <v>-0.163478264136423</v>
       </c>
       <c r="L228" t="n">
         <v>0.0112179112527027</v>
@@ -22791,31 +22791,31 @@
         <v>-0.000331243183112972</v>
       </c>
       <c r="W228" t="n">
-        <v>0.0380058951204738</v>
+        <v>0.0973185863976518</v>
       </c>
       <c r="X228" t="n">
-        <v>0.0167627773070017</v>
+        <v>0.018809714516209</v>
       </c>
       <c r="Y228" t="n">
-        <v>-0.177038582156692</v>
+        <v>-0.105730073570082</v>
       </c>
       <c r="Z228" t="n">
         <v>-0.152531594667403</v>
       </c>
       <c r="AA228" t="n">
-        <v>0.230241981603341</v>
+        <v>0.204613883045715</v>
       </c>
       <c r="AB228" t="n">
-        <v>-0.13425725627333</v>
+        <v>-0.0724148963587344</v>
       </c>
       <c r="AC228" t="n">
-        <v>0.0963138581444369</v>
+        <v>0.132356762228991</v>
       </c>
       <c r="AD228" t="n">
-        <v>-0.233256318679658</v>
+        <v>-0.125904906008493</v>
       </c>
       <c r="AE228" t="n">
-        <v>-0.516201801892465</v>
+        <v>-0.361142960158199</v>
       </c>
     </row>
     <row r="229">
@@ -22829,19 +22829,19 @@
         <v>0</v>
       </c>
       <c r="D229" t="n">
-        <v>-0.0740335034467193</v>
+        <v>-0.165116319891259</v>
       </c>
       <c r="E229" t="n">
         <v>-0.197899650539364</v>
       </c>
       <c r="F229" t="n">
-        <v>0.18590347471302</v>
+        <v>0.107630730154888</v>
       </c>
       <c r="G229" t="n">
         <v>0.0204160513133088</v>
       </c>
       <c r="H229" t="n">
-        <v>-0.00296158508503321</v>
+        <v>0.0493861343210963</v>
       </c>
       <c r="I229" t="n">
         <v>-0.053079148925832</v>
@@ -22850,7 +22850,7 @@
         <v>0.0067193024769731</v>
       </c>
       <c r="K229" t="n">
-        <v>-0.119380942769053</v>
+        <v>-0.113637191433968</v>
       </c>
       <c r="L229" t="n">
         <v>0.0113523493807398</v>
@@ -22886,31 +22886,31 @@
         <v>-0.000325851368956437</v>
       </c>
       <c r="W229" t="n">
-        <v>0.0329654654605226</v>
+        <v>0.063561203381111</v>
       </c>
       <c r="X229" t="n">
-        <v>0.0109291482009957</v>
+        <v>0.000018152870251071</v>
       </c>
       <c r="Y229" t="n">
-        <v>-0.133633157475139</v>
+        <v>-0.224715973919679</v>
       </c>
       <c r="Z229" t="n">
         <v>-0.138299996510944</v>
       </c>
       <c r="AA229" t="n">
-        <v>0.157068170398966</v>
+        <v>0.131073674303589</v>
       </c>
       <c r="AB229" t="n">
-        <v>-0.088895039554173</v>
+        <v>-0.0634380142755315</v>
       </c>
       <c r="AC229" t="n">
-        <v>0.0683214224166084</v>
+        <v>0.0677239711369383</v>
       </c>
       <c r="AD229" t="n">
-        <v>-0.203611731569474</v>
+        <v>-0.295291999293684</v>
       </c>
       <c r="AE229" t="n">
-        <v>-0.304625398459499</v>
+        <v>-0.243284718589681</v>
       </c>
     </row>
     <row r="230">
@@ -22924,19 +22924,19 @@
         <v>0</v>
       </c>
       <c r="D230" t="n">
-        <v>-0.156646793912529</v>
+        <v>-0.162254675936471</v>
       </c>
       <c r="E230" t="n">
         <v>-0.20211764350637</v>
       </c>
       <c r="F230" t="n">
-        <v>0.0508575201017416</v>
+        <v>0.0139635545307985</v>
       </c>
       <c r="G230" t="n">
         <v>0.0212613884524714</v>
       </c>
       <c r="H230" t="n">
-        <v>-0.00348616401094434</v>
+        <v>0.0425303234823068</v>
       </c>
       <c r="I230" t="n">
         <v>-0.201670898709106</v>
@@ -22945,7 +22945,7 @@
         <v>0.00826628957641573</v>
       </c>
       <c r="K230" t="n">
-        <v>-0.114471191068539</v>
+        <v>-0.10293882747997</v>
       </c>
       <c r="L230" t="n">
         <v>0.0116439678568133</v>
@@ -22981,31 +22981,31 @@
         <v>-0.000319965038080787</v>
       </c>
       <c r="W230" t="n">
-        <v>0.0339260078475304</v>
+        <v>0.072466915230067</v>
       </c>
       <c r="X230" t="n">
-        <v>0.000739155310379238</v>
+        <v>-0.00628702681993144</v>
       </c>
       <c r="Y230" t="n">
-        <v>-0.202100960212546</v>
+        <v>-0.207708842236488</v>
       </c>
       <c r="Z230" t="n">
         <v>-0.156663477206352</v>
       </c>
       <c r="AA230" t="n">
-        <v>-0.124622310397659</v>
+        <v>-0.115491337879815</v>
       </c>
       <c r="AB230" t="n">
-        <v>-0.0857868419474303</v>
+        <v>-0.042701741532919</v>
       </c>
       <c r="AC230" t="n">
-        <v>-0.210522469371586</v>
+        <v>-0.158245356785274</v>
       </c>
       <c r="AD230" t="n">
-        <v>-0.569286906790484</v>
+        <v>-0.522617676228115</v>
       </c>
       <c r="AE230" t="n">
-        <v>-0.242541307644678</v>
+        <v>-0.229250642076623</v>
       </c>
     </row>
     <row r="231">
@@ -23019,19 +23019,19 @@
         <v>0</v>
       </c>
       <c r="D231" t="n">
-        <v>-6.35462787190733</v>
+        <v>-6.4825650475632</v>
       </c>
       <c r="E231" t="n">
         <v>-10.9180831107143</v>
       </c>
       <c r="F231" t="n">
-        <v>7.24994277935586</v>
+        <v>7.3288722138594</v>
       </c>
       <c r="G231" t="n">
         <v>4.14303025462738</v>
       </c>
       <c r="H231" t="n">
-        <v>0.23620144879535</v>
+        <v>0.229761288016204</v>
       </c>
       <c r="I231" t="n">
         <v>-1.89348158907485</v>
@@ -23040,7 +23040,7 @@
         <v>0.0782687667864247</v>
       </c>
       <c r="K231" t="n">
-        <v>-7.12204386013532</v>
+        <v>-7.11574623799763</v>
       </c>
       <c r="L231" t="n">
         <v>-0.731684035695398</v>
@@ -23076,31 +23076,31 @@
         <v>-0.000252815883905431</v>
       </c>
       <c r="W231" t="n">
-        <v>-5.94385772904819</v>
+        <v>-5.99448737624325</v>
       </c>
       <c r="X231" t="n">
-        <v>-0.975314053476406</v>
+        <v>-0.971539615826814</v>
       </c>
       <c r="Y231" t="n">
-        <v>-7.96055002868393</v>
+        <v>-8.0884872043398</v>
       </c>
       <c r="Z231" t="n">
         <v>-9.31216095393765</v>
       </c>
       <c r="AA231" t="n">
-        <v>9.68228748089152</v>
+        <v>9.75315307695071</v>
       </c>
       <c r="AB231" t="n">
-        <v>-15.6596127135263</v>
+        <v>-15.7038412508325</v>
       </c>
       <c r="AC231" t="n">
-        <v>-4.3735060256683</v>
+        <v>-4.33043574264703</v>
       </c>
       <c r="AD231" t="n">
-        <v>-21.6462170082899</v>
+        <v>-21.7310839009245</v>
       </c>
       <c r="AE231" t="n">
-        <v>-5.66309299133237</v>
+        <v>-5.66872462061369</v>
       </c>
     </row>
     <row r="232">
@@ -23120,13 +23120,13 @@
         <v>#NUM!</v>
       </c>
       <c r="F232" t="n">
-        <v>7.24061874705758</v>
+        <v>7.30017600255913</v>
       </c>
       <c r="G232" t="n">
         <v>4.10363982228423</v>
       </c>
       <c r="H232" t="n">
-        <v>0.231610770995828</v>
+        <v>0.225264301357652</v>
       </c>
       <c r="I232" t="n">
         <v>0</v>
@@ -23135,7 +23135,7 @@
         <v>0.0762012506659499</v>
       </c>
       <c r="K232" t="n">
-        <v>-6.99714711879506</v>
+        <v>-6.99701386962174</v>
       </c>
       <c r="L232" t="n">
         <v>-0.727705117698837</v>
@@ -23171,10 +23171,10 @@
         <v>-0.000247948531799295</v>
       </c>
       <c r="W232" t="n">
-        <v>-5.90258800606652</v>
+        <v>-5.96375327479904</v>
       </c>
       <c r="X232" t="n">
-        <v>-0.965707748995162</v>
+        <v>-0.966809286720248</v>
       </c>
       <c r="Y232" t="e">
         <v>#NUM!</v>
@@ -23183,19 +23183,19 @@
         <v>#NUM!</v>
       </c>
       <c r="AA232" t="n">
-        <v>11.2916002369718</v>
+        <v>11.3426905019546</v>
       </c>
       <c r="AB232" t="n">
-        <v>-15.432317162843</v>
+        <v>-15.5002515805719</v>
       </c>
       <c r="AC232" t="n">
-        <v>-2.28876978830089</v>
+        <v>-2.2890309171096</v>
       </c>
       <c r="AD232" t="n">
         <v>0</v>
       </c>
       <c r="AE232" t="n">
-        <v>-5.60477891166246</v>
+        <v>-5.63724839411157</v>
       </c>
     </row>
     <row r="233">
@@ -23215,13 +23215,13 @@
         <v>#NUM!</v>
       </c>
       <c r="F233" t="n">
-        <v>3.70012666585979</v>
+        <v>3.70383543718708</v>
       </c>
       <c r="G233" t="n">
         <v>2.06381297055394</v>
       </c>
       <c r="H233" t="n">
-        <v>0.235503788278021</v>
+        <v>0.229234156125654</v>
       </c>
       <c r="I233" t="n">
         <v>0</v>
@@ -23230,7 +23230,7 @@
         <v>0.0755541209685337</v>
       </c>
       <c r="K233" t="n">
-        <v>-6.88000796891369</v>
+        <v>-6.86747435479228</v>
       </c>
       <c r="L233" t="n">
         <v>-0.725077670364884</v>
@@ -23266,10 +23266,10 @@
         <v>-0.000243588812998019</v>
       </c>
       <c r="W233" t="n">
-        <v>-5.8642497312584</v>
+        <v>-5.90629203205199</v>
       </c>
       <c r="X233" t="n">
-        <v>-0.954076810292782</v>
+        <v>-0.947120950463217</v>
       </c>
       <c r="Y233" t="e">
         <v>#NUM!</v>
@@ -23278,19 +23278,19 @@
         <v>#NUM!</v>
       </c>
       <c r="AA233" t="n">
-        <v>5.97363300303747</v>
+        <v>5.9713656487234</v>
       </c>
       <c r="AB233" t="n">
-        <v>-15.232345854173</v>
+        <v>-15.2566839896174</v>
       </c>
       <c r="AC233" t="n">
-        <v>-8.30296838048652</v>
+        <v>-8.32844959134408</v>
       </c>
       <c r="AD233" t="n">
         <v>0</v>
       </c>
       <c r="AE233" t="n">
-        <v>-5.55387597877009</v>
+        <v>-5.56342539428815</v>
       </c>
     </row>
     <row r="234">
@@ -23310,13 +23310,13 @@
         <v>#NUM!</v>
       </c>
       <c r="F234" t="n">
-        <v>3.54124599920147</v>
+        <v>3.6190399799111</v>
       </c>
       <c r="G234" t="n">
         <v>2.04452940303916</v>
       </c>
       <c r="H234" t="n">
-        <v>0.23443383822375</v>
+        <v>0.228250090588388</v>
       </c>
       <c r="I234" t="n">
         <v>0</v>
@@ -23325,7 +23325,7 @@
         <v>0.0785155806756128</v>
       </c>
       <c r="K234" t="n">
-        <v>-6.88177678056897</v>
+        <v>-6.88148463390872</v>
       </c>
       <c r="L234" t="n">
         <v>-0.722042677932606</v>
@@ -23361,10 +23361,10 @@
         <v>-0.000239129527510748</v>
       </c>
       <c r="W234" t="n">
-        <v>-5.82271178477694</v>
+        <v>-5.8832342610377</v>
       </c>
       <c r="X234" t="n">
-        <v>-0.941958385820405</v>
+        <v>-0.943430367024577</v>
       </c>
       <c r="Y234" t="e">
         <v>#NUM!</v>
@@ -23373,19 +23373,19 @@
         <v>#NUM!</v>
       </c>
       <c r="AA234" t="n">
-        <v>5.80219913243003</v>
+        <v>5.87220670973692</v>
       </c>
       <c r="AB234" t="n">
-        <v>-15.1625964650592</v>
+        <v>-15.2299649666933</v>
       </c>
       <c r="AC234" t="n">
-        <v>-8.43731193228799</v>
+        <v>-8.41934981094317</v>
       </c>
       <c r="AD234" t="n">
         <v>0</v>
       </c>
       <c r="AE234" t="n">
-        <v>-5.41155425207247</v>
+        <v>-5.43277097523112</v>
       </c>
     </row>
     <row r="235">
@@ -23405,13 +23405,13 @@
         <v>#NUM!</v>
       </c>
       <c r="F235" t="n">
-        <v>3.49547887778444</v>
+        <v>3.57214368642037</v>
       </c>
       <c r="G235" t="n">
         <v>2.02312068909619</v>
       </c>
       <c r="H235" t="n">
-        <v>0.236866424865927</v>
+        <v>0.230756391199535</v>
       </c>
       <c r="I235" t="n">
         <v>0</v>
@@ -23468,19 +23468,19 @@
         <v>#NUM!</v>
       </c>
       <c r="AA235" t="n">
-        <v>5.73691017249106</v>
+        <v>5.80589854628874</v>
       </c>
       <c r="AB235" t="n">
         <v>-0.0860268363079363</v>
       </c>
       <c r="AC235" t="n">
-        <v>5.65619406006092</v>
+        <v>5.72524699647437</v>
       </c>
       <c r="AD235" t="n">
         <v>0</v>
       </c>
       <c r="AE235" t="n">
-        <v>0</v>
+        <v>0.000000000000000888178419700125</v>
       </c>
     </row>
     <row r="236">
@@ -23500,13 +23500,13 @@
         <v>#NUM!</v>
       </c>
       <c r="F236" t="n">
-        <v>3.45732600778049</v>
+        <v>3.53302887178381</v>
       </c>
       <c r="G236" t="n">
         <v>2.00423722863772</v>
       </c>
       <c r="H236" t="n">
-        <v>0.239850512193163</v>
+        <v>0.0722448881001593</v>
       </c>
       <c r="I236" t="n">
         <v>0</v>
@@ -23563,19 +23563,19 @@
         <v>#NUM!</v>
       </c>
       <c r="AA236" t="n">
-        <v>5.68335162943522</v>
+        <v>5.59952103983218</v>
       </c>
       <c r="AB236" t="n">
         <v>-0.0651868979666943</v>
       </c>
       <c r="AC236" t="n">
-        <v>5.62214522412064</v>
+        <v>5.53825530337416</v>
       </c>
       <c r="AD236" t="n">
         <v>0</v>
       </c>
       <c r="AE236" t="n">
-        <v>0</v>
+        <v>0.000000000000000888178419700125</v>
       </c>
     </row>
     <row r="237">
@@ -23595,13 +23595,13 @@
         <v>#NUM!</v>
       </c>
       <c r="F237" t="n">
-        <v>3.41595841441796</v>
+        <v>3.49062824628225</v>
       </c>
       <c r="G237" t="n">
         <v>1.98462400626479</v>
       </c>
       <c r="H237" t="n">
-        <v>0.233993888858739</v>
+        <v>0.0705331289343471</v>
       </c>
       <c r="I237" t="n">
         <v>0</v>
@@ -23658,19 +23658,19 @@
         <v>#NUM!</v>
       </c>
       <c r="AA237" t="n">
-        <v>5.61736492486516</v>
+        <v>5.53633467011732</v>
       </c>
       <c r="AB237" t="n">
         <v>-0.0649308917620592</v>
       </c>
       <c r="AC237" t="n">
-        <v>5.55635070803114</v>
+        <v>5.47526336804371</v>
       </c>
       <c r="AD237" t="n">
         <v>0</v>
       </c>
       <c r="AE237" t="n">
-        <v>0</v>
+        <v>0.000000000000000888178419700125</v>
       </c>
     </row>
     <row r="238">
@@ -23690,13 +23690,13 @@
         <v>#NUM!</v>
       </c>
       <c r="F238" t="n">
-        <v>3.4627109495069</v>
+        <v>3.51824978588587</v>
       </c>
       <c r="G238" t="n">
         <v>1.96748284330751</v>
       </c>
       <c r="H238" t="n">
-        <v>0.228418237905961</v>
+        <v>0.171482084754022</v>
       </c>
       <c r="I238" t="n">
         <v>0</v>
@@ -23753,19 +23753,19 @@
         <v>#NUM!</v>
       </c>
       <c r="AA238" t="n">
-        <v>5.64022383642352</v>
+        <v>5.64081814717383</v>
       </c>
       <c r="AB238" t="n">
         <v>-0.0608745265794686</v>
       </c>
       <c r="AC238" t="n">
-        <v>5.58303129663076</v>
+        <v>5.58362599945893</v>
       </c>
       <c r="AD238" t="n">
         <v>0</v>
       </c>
       <c r="AE238" t="n">
-        <v>0</v>
+        <v>0.000000000000000888178419700125</v>
       </c>
     </row>
     <row r="239">
@@ -23791,7 +23791,7 @@
         <v>0</v>
       </c>
       <c r="H239" t="n">
-        <v>0.222817251186129</v>
+        <v>0.167276436644511</v>
       </c>
       <c r="I239" t="n">
         <v>0</v>
@@ -23848,19 +23848,19 @@
         <v>#NUM!</v>
       </c>
       <c r="AA239" t="n">
-        <v>0.293502538494835</v>
+        <v>0.238003495894634</v>
       </c>
       <c r="AB239" t="n">
         <v>-0.0335228701561467</v>
       </c>
       <c r="AC239" t="n">
-        <v>0.260084071600606</v>
+        <v>0.204565278828774</v>
       </c>
       <c r="AD239" t="n">
         <v>0</v>
       </c>
       <c r="AE239" t="n">
-        <v>0</v>
+        <v>0.000000000000000888178419700125</v>
       </c>
     </row>
     <row r="240">
@@ -23886,7 +23886,7 @@
         <v>0</v>
       </c>
       <c r="H240" t="n">
-        <v>0.217095225343289</v>
+        <v>0.162979900079402</v>
       </c>
       <c r="I240" t="n">
         <v>0</v>
@@ -23943,19 +23943,19 @@
         <v>#NUM!</v>
       </c>
       <c r="AA240" t="n">
-        <v>0.286316467813129</v>
+        <v>0.232241012889103</v>
       </c>
       <c r="AB240" t="n">
         <v>-0.0327638569113506</v>
       </c>
       <c r="AC240" t="n">
-        <v>0.25365219250096</v>
+        <v>0.199557922250519</v>
       </c>
       <c r="AD240" t="n">
         <v>0</v>
       </c>
       <c r="AE240" t="n">
-        <v>0</v>
+        <v>0.000000000000000888178419700125</v>
       </c>
     </row>
     <row r="241">
@@ -23981,7 +23981,7 @@
         <v>0</v>
       </c>
       <c r="H241" t="n">
-        <v>0.211680444347253</v>
+        <v>0.158914143637246</v>
       </c>
       <c r="I241" t="n">
         <v>0</v>
@@ -24038,19 +24038,19 @@
         <v>#NUM!</v>
       </c>
       <c r="AA241" t="n">
-        <v>0.279669510502595</v>
+        <v>0.22694137755605</v>
       </c>
       <c r="AB241" t="n">
         <v>-0.0325003623948072</v>
       </c>
       <c r="AC241" t="n">
-        <v>0.247265599956117</v>
+        <v>0.19451927492442</v>
       </c>
       <c r="AD241" t="n">
         <v>0</v>
       </c>
       <c r="AE241" t="n">
-        <v>0</v>
+        <v>0.000000000000000888178419700125</v>
       </c>
     </row>
     <row r="242">
@@ -24076,7 +24076,7 @@
         <v>0</v>
       </c>
       <c r="H242" t="n">
-        <v>0.206544383462085</v>
+        <v>0.15953336701643</v>
       </c>
       <c r="I242" t="n">
         <v>0</v>
@@ -24133,19 +24133,19 @@
         <v>#NUM!</v>
       </c>
       <c r="AA242" t="n">
-        <v>0.273168337399117</v>
+        <v>0.22619059559475</v>
       </c>
       <c r="AB242" t="n">
         <v>-0.0315912555671793</v>
       </c>
       <c r="AC242" t="n">
-        <v>0.241668531528796</v>
+        <v>0.194675056494781</v>
       </c>
       <c r="AD242" t="n">
         <v>0</v>
       </c>
       <c r="AE242" t="n">
-        <v>0</v>
+        <v>0.000000000000000888178419700125</v>
       </c>
     </row>
     <row r="243">
@@ -24240,7 +24240,7 @@
         <v>0</v>
       </c>
       <c r="AE243" t="n">
-        <v>0</v>
+        <v>0.000000000000000888178419700125</v>
       </c>
     </row>
     <row r="244">
@@ -24335,7 +24335,7 @@
         <v>0</v>
       </c>
       <c r="AE244" t="n">
-        <v>0</v>
+        <v>0.000000000000000888178419700125</v>
       </c>
     </row>
     <row r="245">
@@ -24430,7 +24430,7 @@
         <v>0</v>
       </c>
       <c r="AE245" t="n">
-        <v>0</v>
+        <v>0.000000000000000888178419700125</v>
       </c>
     </row>
     <row r="246">
@@ -24525,7 +24525,7 @@
         <v>0</v>
       </c>
       <c r="AE246" t="n">
-        <v>0</v>
+        <v>0.000000000000000888178419700125</v>
       </c>
     </row>
     <row r="247">
@@ -24620,7 +24620,7 @@
         <v>0</v>
       </c>
       <c r="AE247" t="n">
-        <v>0</v>
+        <v>0.000000000000000888178419700125</v>
       </c>
     </row>
     <row r="248">
@@ -24715,7 +24715,7 @@
         <v>0</v>
       </c>
       <c r="AE248" t="n">
-        <v>0</v>
+        <v>0.000000000000000888178419700125</v>
       </c>
     </row>
     <row r="249">
@@ -24810,7 +24810,7 @@
         <v>0</v>
       </c>
       <c r="AE249" t="n">
-        <v>0</v>
+        <v>0.000000000000000888178419700125</v>
       </c>
     </row>
     <row r="250">
@@ -24905,7 +24905,7 @@
         <v>0</v>
       </c>
       <c r="AE250" t="n">
-        <v>0</v>
+        <v>0.000000000000000888178419700125</v>
       </c>
     </row>
     <row r="251">
@@ -25000,7 +25000,7 @@
         <v>0</v>
       </c>
       <c r="AE251" t="n">
-        <v>0</v>
+        <v>0.000000000000000888178419700125</v>
       </c>
     </row>
     <row r="252">
@@ -25095,7 +25095,7 @@
         <v>0</v>
       </c>
       <c r="AE252" t="n">
-        <v>0</v>
+        <v>0.000000000000000888178419700125</v>
       </c>
     </row>
     <row r="253">
@@ -25190,7 +25190,7 @@
         <v>0</v>
       </c>
       <c r="AE253" t="n">
-        <v>0</v>
+        <v>0.000000000000000888178419700125</v>
       </c>
     </row>
     <row r="254">
@@ -25285,7 +25285,7 @@
         <v>0</v>
       </c>
       <c r="AE254" t="n">
-        <v>0</v>
+        <v>0.000000000000000888178419700125</v>
       </c>
     </row>
     <row r="255">
@@ -25380,7 +25380,7 @@
         <v>0</v>
       </c>
       <c r="AE255" t="n">
-        <v>0</v>
+        <v>0.000000000000000888178419700125</v>
       </c>
     </row>
     <row r="256">
@@ -25475,7 +25475,7 @@
         <v>0</v>
       </c>
       <c r="AE256" t="n">
-        <v>0</v>
+        <v>0.000000000000000888178419700125</v>
       </c>
     </row>
     <row r="257">
@@ -25570,7 +25570,7 @@
         <v>0</v>
       </c>
       <c r="AE257" t="n">
-        <v>0</v>
+        <v>0.000000000000000888178419700125</v>
       </c>
     </row>
     <row r="258">
@@ -25665,7 +25665,7 @@
         <v>0</v>
       </c>
       <c r="AE258" t="n">
-        <v>0</v>
+        <v>0.000000000000000888178419700125</v>
       </c>
     </row>
     <row r="259">
@@ -25760,7 +25760,7 @@
         <v>0</v>
       </c>
       <c r="AE259" t="n">
-        <v>0</v>
+        <v>0.000000000000000888178419700125</v>
       </c>
     </row>
     <row r="260">
@@ -25855,7 +25855,7 @@
         <v>0</v>
       </c>
       <c r="AE260" t="n">
-        <v>0</v>
+        <v>0.000000000000000888178419700125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>